<commit_message>
Add aba de pedidos por cidade do Triângulo Mineiro/Alto Paranaíba
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015qQhQ5WL7n1bFV4ZTWbMQc
</commit_message>
<xml_diff>
--- a/volumetria_pedidos_estado_capitais.xlsx
+++ b/volumetria_pedidos_estado_capitais.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Por Estado" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Capitais" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Triângulo Mineiro" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1420,9 +1421,956 @@
       <c r="C29" t="n">
         <v>15084</v>
       </c>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="n">
         <v>31.2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Cidade</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Microrregião</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Região</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Pedidos</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Cancelados</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>% da região</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Uberlândia</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Uberlândia</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Triângulo Mineiro</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>76</v>
+      </c>
+      <c r="E2" t="n">
+        <v>7</v>
+      </c>
+      <c r="F2" t="n">
+        <v>29.8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Uberaba</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Uberaba</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Triângulo Mineiro</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>52</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>20.4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Patos de Minas</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Patos de Minas</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Alto Paranaíba</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>28</v>
+      </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Araguari</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Uberlândia</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Triângulo Mineiro</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>13</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>5.1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Patrocínio</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Patrocínio</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Alto Paranaíba</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>13</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>5.1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Araxá</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Araxá</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Alto Paranaíba</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>11</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ituiutaba</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Ituiutaba</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Triângulo Mineiro</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>11</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>São Gotardo</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Patos de Minas</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Alto Paranaíba</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Carmo do Paranaíba</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Patos de Minas</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Alto Paranaíba</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Frutal</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Frutal</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Triângulo Mineiro</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Sacramento</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Araxá</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Alto Paranaíba</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Prata</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Uberlândia</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Triângulo Mineiro</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Coromandel</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Patrocínio</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Alto Paranaíba</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Veríssimo</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Uberaba</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Triângulo Mineiro</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Lagoa Formosa</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Patos de Minas</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Alto Paranaíba</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Iraí de Minas</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Patrocínio</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Alto Paranaíba</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Campos Altos</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Araxá</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Alto Paranaíba</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Iturama</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Frutal</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Triângulo Mineiro</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Araporã</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Uberlândia</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Triângulo Mineiro</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Conceição das Alagoas</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Uberaba</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Triângulo Mineiro</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Capinópolis</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Ituiutaba</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Triângulo Mineiro</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Delta</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Uberaba</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Triângulo Mineiro</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Campina Verde</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Frutal</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Triângulo Mineiro</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Canápolis</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Uberlândia</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Triângulo Mineiro</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Centralina</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Uberlândia</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Triângulo Mineiro</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Arapuá</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Patos de Minas</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Alto Paranaíba</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Rio Paranaíba</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Patos de Minas</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Alto Paranaíba</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Perdizes</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Araxá</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Alto Paranaíba</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Pedrinópolis</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Araxá</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Alto Paranaíba</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Monte Carmelo</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Patrocínio</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Alto Paranaíba</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Nova Ponte</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Araxá</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Alto Paranaíba</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Santa Vitória</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Ituiutaba</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Triângulo Mineiro</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Serra do Salitre</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Patrocínio</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Alto Paranaíba</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Tupaciguara</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Uberlândia</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Triângulo Mineiro</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="n">
+        <v>255</v>
+      </c>
+      <c r="E36" t="n">
+        <v>15</v>
+      </c>
+      <c r="F36" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>